<commit_message>
fix: professional workbook formatting across all models
Sensitivity grids/stats render whole currency; WACC betas 0.00 and
costs of equity as percent; zero premiums explicit 0.00%; cash-flow
detail whole units; Data Review mirrors two decimals; F12 matches
input styling on all scenario sheets; cell comments stripped at the
single export choke point (recalc already dropped them from gated
builds). Guard script enforces 0 violations (306 before). Rebuilt
AAPL/AGNC/XOM/BLK/PFE examples through the gate.
</commit_message>
<xml_diff>
--- a/excel model/2026-10-03_BLK_DCF.xlsx
+++ b/excel model/2026-10-03_BLK_DCF.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Data Review" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Data Review'!$A$5:$I$242</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Data Review'!$A$5:$I$244</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1608" uniqueCount="317">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1612" uniqueCount="319">
   <si>
     <t xml:space="preserve">BlackRock, Inc. (BLK) — AUM and Fee-Driven FCFF Valuation</t>
   </si>
@@ -971,7 +971,13 @@
     <t xml:space="preserve">These fee components are not separately reported in the latest mapped filing and remain visible as source gaps: capital_allocation_income, administrative_other_revenue.</t>
   </si>
   <si>
+    <t xml:space="preserve">financials: data status is cached</t>
+  </si>
+  <si>
     <t xml:space="preserve">valuation_context: data status is cached</t>
+  </si>
+  <si>
+    <t xml:space="preserve">peers: data status is cached</t>
   </si>
   <si>
     <t xml:space="preserve">insider_trades: Insider trades are intentionally lazy-loaded and do not block the primary valuation load.</t>
@@ -981,7 +987,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="8">
+  <numFmts count="9">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* \-??_-;_-@_-"/>
     <numFmt numFmtId="166" formatCode="_-\$* #,##0.00_-;&quot;-$&quot;* #,##0.00_-;_-\$* \-??_-;_-@_-"/>
@@ -990,6 +996,7 @@
     <numFmt numFmtId="169" formatCode="0.0%;[RED]\(0.0%\);0.0%"/>
     <numFmt numFmtId="170" formatCode="0.000\x"/>
     <numFmt numFmtId="171" formatCode="\$#,##0.00;[RED]&quot;($&quot;#,##0.00\);\-"/>
+    <numFmt numFmtId="172" formatCode="#,##0.00"/>
   </numFmts>
   <fonts count="24">
     <font>
@@ -1359,7 +1366,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1449,6 +1456,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4060,7 +4071,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I242"/>
+  <dimension ref="A1:I244"/>
   <sheetFormatPr defaultColWidth="8.73828125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -4139,7 +4150,7 @@
       <c r="C6" s="22" t="s">
         <v>131</v>
       </c>
-      <c r="D6" s="22" t="n">
+      <c r="D6" s="23" t="n">
         <v>10008995000000</v>
       </c>
       <c r="E6" s="22" t="s">
@@ -4168,7 +4179,7 @@
       <c r="C7" s="22" t="s">
         <v>137</v>
       </c>
-      <c r="D7" s="22" t="n">
+      <c r="D7" s="23" t="n">
         <v>8594485000000</v>
       </c>
       <c r="E7" s="22" t="s">
@@ -4197,7 +4208,7 @@
       <c r="C8" s="22" t="s">
         <v>139</v>
       </c>
-      <c r="D8" s="22" t="n">
+      <c r="D8" s="23" t="n">
         <v>9301740000000</v>
       </c>
       <c r="E8" s="22" t="s">
@@ -4226,7 +4237,7 @@
       <c r="C9" s="22" t="s">
         <v>139</v>
       </c>
-      <c r="D9" s="22" t="n">
+      <c r="D9" s="23" t="n">
         <v>9301740000000</v>
       </c>
       <c r="E9" s="22" t="s">
@@ -4255,7 +4266,7 @@
       <c r="C10" s="22" t="s">
         <v>140</v>
       </c>
-      <c r="D10" s="22" t="n">
+      <c r="D10" s="23" t="n">
         <v>288695000000</v>
       </c>
       <c r="E10" s="22" t="s">
@@ -4305,7 +4316,7 @@
       <c r="C12" s="22" t="s">
         <v>149</v>
       </c>
-      <c r="D12" s="22" t="n">
+      <c r="D12" s="23" t="n">
         <v>2177000000</v>
       </c>
       <c r="E12" s="22" t="s">
@@ -4334,7 +4345,7 @@
       <c r="C13" s="22" t="s">
         <v>152</v>
       </c>
-      <c r="D13" s="22" t="n">
+      <c r="D13" s="23" t="n">
         <v>1073550000000</v>
       </c>
       <c r="E13" s="22" t="s">
@@ -4363,7 +4374,7 @@
       <c r="C14" s="22" t="s">
         <v>155</v>
       </c>
-      <c r="D14" s="22" t="n">
+      <c r="D14" s="23" t="n">
         <v>50088000000</v>
       </c>
       <c r="E14" s="22" t="s">
@@ -4392,7 +4403,7 @@
       <c r="C15" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="D15" s="22" t="n">
+      <c r="D15" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E15" s="22" t="s">
@@ -4421,7 +4432,7 @@
       <c r="C16" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="D16" s="22" t="n">
+      <c r="D16" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E16" s="22" t="s">
@@ -4450,7 +4461,7 @@
       <c r="C17" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="D17" s="22" t="n">
+      <c r="D17" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E17" s="22" t="s">
@@ -4479,7 +4490,7 @@
       <c r="C18" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="D18" s="22" t="n">
+      <c r="D18" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E18" s="22" t="s">
@@ -4508,7 +4519,7 @@
       <c r="C19" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="D19" s="22" t="n">
+      <c r="D19" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E19" s="22" t="s">
@@ -4537,7 +4548,7 @@
       <c r="C20" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="D20" s="22" t="n">
+      <c r="D20" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E20" s="22" t="s">
@@ -4566,7 +4577,7 @@
       <c r="C21" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="D21" s="22" t="n">
+      <c r="D21" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E21" s="22" t="s">
@@ -4595,7 +4606,7 @@
       <c r="C22" s="22" t="s">
         <v>168</v>
       </c>
-      <c r="D22" s="22" t="n">
+      <c r="D22" s="23" t="n">
         <v>427000000</v>
       </c>
       <c r="E22" s="22" t="s">
@@ -4645,7 +4656,7 @@
       <c r="C24" s="22" t="s">
         <v>173</v>
       </c>
-      <c r="D24" s="22" t="n">
+      <c r="D24" s="23" t="n">
         <v>346000000</v>
       </c>
       <c r="E24" s="22" t="s">
@@ -4674,7 +4685,7 @@
       <c r="C25" s="22" t="s">
         <v>173</v>
       </c>
-      <c r="D25" s="22" t="n">
+      <c r="D25" s="23" t="n">
         <v>346000000</v>
       </c>
       <c r="E25" s="22" t="s">
@@ -4703,7 +4714,7 @@
       <c r="C26" s="22" t="s">
         <v>173</v>
       </c>
-      <c r="D26" s="22" t="n">
+      <c r="D26" s="23" t="n">
         <v>346000000</v>
       </c>
       <c r="E26" s="22" t="s">
@@ -4732,7 +4743,7 @@
       <c r="C27" s="22" t="s">
         <v>173</v>
       </c>
-      <c r="D27" s="22" t="n">
+      <c r="D27" s="23" t="n">
         <v>346000000</v>
       </c>
       <c r="E27" s="22" t="s">
@@ -4761,7 +4772,7 @@
       <c r="C28" s="22" t="s">
         <v>173</v>
       </c>
-      <c r="D28" s="22" t="n">
+      <c r="D28" s="23" t="n">
         <v>346000000</v>
       </c>
       <c r="E28" s="22" t="s">
@@ -4790,7 +4801,7 @@
       <c r="C29" s="22" t="s">
         <v>173</v>
       </c>
-      <c r="D29" s="22" t="n">
+      <c r="D29" s="23" t="n">
         <v>346000000</v>
       </c>
       <c r="E29" s="22" t="s">
@@ -4819,7 +4830,7 @@
       <c r="C30" s="22" t="s">
         <v>173</v>
       </c>
-      <c r="D30" s="22" t="n">
+      <c r="D30" s="23" t="n">
         <v>346000000</v>
       </c>
       <c r="E30" s="22" t="s">
@@ -4848,7 +4859,7 @@
       <c r="C31" s="22" t="s">
         <v>188</v>
       </c>
-      <c r="D31" s="22" t="n">
+      <c r="D31" s="23" t="n">
         <v>13724000000</v>
       </c>
       <c r="E31" s="22" t="s">
@@ -4985,7 +4996,7 @@
       <c r="C36" s="22" t="s">
         <v>194</v>
       </c>
-      <c r="D36" s="22" t="n">
+      <c r="D36" s="23" t="n">
         <v>554000000</v>
       </c>
       <c r="E36" s="22" t="s">
@@ -5014,7 +5025,7 @@
       <c r="C37" s="22" t="s">
         <v>196</v>
       </c>
-      <c r="D37" s="22" t="n">
+      <c r="D37" s="23" t="n">
         <v>675000000</v>
       </c>
       <c r="E37" s="22" t="s">
@@ -5043,7 +5054,7 @@
       <c r="C38" s="22" t="s">
         <v>198</v>
       </c>
-      <c r="D38" s="22" t="n">
+      <c r="D38" s="23" t="n">
         <v>1485000000</v>
       </c>
       <c r="E38" s="22" t="s">
@@ -5072,7 +5083,7 @@
       <c r="C39" s="22" t="s">
         <v>200</v>
       </c>
-      <c r="D39" s="22" t="n">
+      <c r="D39" s="23" t="n">
         <v>1262000000</v>
       </c>
       <c r="E39" s="22" t="s">
@@ -5122,7 +5133,7 @@
       <c r="C41" s="22" t="s">
         <v>204</v>
       </c>
-      <c r="D41" s="22" t="n">
+      <c r="D41" s="23" t="n">
         <v>159000000</v>
       </c>
       <c r="E41" s="22" t="s">
@@ -5151,7 +5162,7 @@
       <c r="C42" s="22" t="s">
         <v>206</v>
       </c>
-      <c r="D42" s="22" t="n">
+      <c r="D42" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E42" s="22" t="s">
@@ -5180,7 +5191,7 @@
       <c r="C43" s="22" t="s">
         <v>206</v>
       </c>
-      <c r="D43" s="22" t="n">
+      <c r="D43" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E43" s="22" t="s">
@@ -5209,7 +5220,7 @@
       <c r="C44" s="22" t="s">
         <v>206</v>
       </c>
-      <c r="D44" s="22" t="n">
+      <c r="D44" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E44" s="22" t="s">
@@ -5238,7 +5249,7 @@
       <c r="C45" s="22" t="s">
         <v>206</v>
       </c>
-      <c r="D45" s="22" t="n">
+      <c r="D45" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E45" s="22" t="s">
@@ -5267,7 +5278,7 @@
       <c r="C46" s="22" t="s">
         <v>206</v>
       </c>
-      <c r="D46" s="22" t="n">
+      <c r="D46" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E46" s="22" t="s">
@@ -5296,7 +5307,7 @@
       <c r="C47" s="22" t="s">
         <v>206</v>
       </c>
-      <c r="D47" s="22" t="n">
+      <c r="D47" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E47" s="22" t="s">
@@ -5325,7 +5336,7 @@
       <c r="C48" s="22" t="s">
         <v>206</v>
       </c>
-      <c r="D48" s="22" t="n">
+      <c r="D48" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E48" s="22" t="s">
@@ -5354,7 +5365,7 @@
       <c r="C49" s="22" t="s">
         <v>210</v>
       </c>
-      <c r="D49" s="22" t="n">
+      <c r="D49" s="23" t="n">
         <v>17859000000</v>
       </c>
       <c r="E49" s="22" t="s">
@@ -5383,7 +5394,7 @@
       <c r="C50" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="D50" s="22" t="n">
+      <c r="D50" s="23" t="n">
         <v>6275000000</v>
       </c>
       <c r="E50" s="22" t="s">
@@ -5412,7 +5423,7 @@
       <c r="C51" s="22" t="s">
         <v>212</v>
       </c>
-      <c r="D51" s="22" t="n">
+      <c r="D51" s="23" t="n">
         <v>292000000</v>
       </c>
       <c r="E51" s="22" t="s">
@@ -5441,7 +5452,7 @@
       <c r="C52" s="22" t="s">
         <v>214</v>
       </c>
-      <c r="D52" s="22" t="n">
+      <c r="D52" s="23" t="n">
         <v>0.206708595387841</v>
       </c>
       <c r="E52" s="22" t="s">
@@ -5470,7 +5481,7 @@
       <c r="C53" s="22" t="s">
         <v>214</v>
       </c>
-      <c r="D53" s="22" t="n">
+      <c r="D53" s="23" t="n">
         <v>0.206708595387841</v>
       </c>
       <c r="E53" s="22" t="s">
@@ -5499,7 +5510,7 @@
       <c r="C54" s="22" t="s">
         <v>217</v>
       </c>
-      <c r="D54" s="22" t="n">
+      <c r="D54" s="23" t="n">
         <v>344000000</v>
       </c>
       <c r="E54" s="22" t="s">
@@ -5528,7 +5539,7 @@
       <c r="C55" s="22" t="s">
         <v>220</v>
       </c>
-      <c r="D55" s="22" t="n">
+      <c r="D55" s="23" t="n">
         <v>8736000000</v>
       </c>
       <c r="E55" s="22" t="s">
@@ -5603,7 +5614,7 @@
       <c r="C58" s="22" t="s">
         <v>227</v>
       </c>
-      <c r="D58" s="22" t="n">
+      <c r="D58" s="23" t="n">
         <v>346000000</v>
       </c>
       <c r="E58" s="22" t="s">
@@ -5632,7 +5643,7 @@
       <c r="C59" s="22" t="s">
         <v>227</v>
       </c>
-      <c r="D59" s="22" t="n">
+      <c r="D59" s="23" t="n">
         <v>346000000</v>
       </c>
       <c r="E59" s="22" t="s">
@@ -5661,7 +5672,7 @@
       <c r="C60" s="22" t="s">
         <v>227</v>
       </c>
-      <c r="D60" s="22" t="n">
+      <c r="D60" s="23" t="n">
         <v>346000000</v>
       </c>
       <c r="E60" s="22" t="s">
@@ -5690,7 +5701,7 @@
       <c r="C61" s="22" t="s">
         <v>227</v>
       </c>
-      <c r="D61" s="22" t="n">
+      <c r="D61" s="23" t="n">
         <v>346000000</v>
       </c>
       <c r="E61" s="22" t="s">
@@ -5719,7 +5730,7 @@
       <c r="C62" s="22" t="s">
         <v>227</v>
       </c>
-      <c r="D62" s="22" t="n">
+      <c r="D62" s="23" t="n">
         <v>346000000</v>
       </c>
       <c r="E62" s="22" t="s">
@@ -5748,7 +5759,7 @@
       <c r="C63" s="22" t="s">
         <v>227</v>
       </c>
-      <c r="D63" s="22" t="n">
+      <c r="D63" s="23" t="n">
         <v>346000000</v>
       </c>
       <c r="E63" s="22" t="s">
@@ -5777,7 +5788,7 @@
       <c r="C64" s="22" t="s">
         <v>227</v>
       </c>
-      <c r="D64" s="22" t="n">
+      <c r="D64" s="23" t="n">
         <v>346000000</v>
       </c>
       <c r="E64" s="22" t="s">
@@ -5806,7 +5817,7 @@
       <c r="C65" s="22" t="s">
         <v>228</v>
       </c>
-      <c r="D65" s="22" t="n">
+      <c r="D65" s="23" t="n">
         <v>427000000</v>
       </c>
       <c r="E65" s="22" t="s">
@@ -5856,7 +5867,7 @@
       <c r="C67" s="22" t="s">
         <v>230</v>
       </c>
-      <c r="D67" s="22" t="n">
+      <c r="D67" s="23" t="n">
         <v>153000000</v>
       </c>
       <c r="E67" s="22" t="s">
@@ -5906,7 +5917,7 @@
       <c r="C69" s="22" t="s">
         <v>235</v>
       </c>
-      <c r="D69" s="22" t="n">
+      <c r="D69" s="23" t="n">
         <v>150706451</v>
       </c>
       <c r="E69" s="22" t="s">
@@ -5935,7 +5946,7 @@
       <c r="C70" s="22" t="s">
         <v>131</v>
       </c>
-      <c r="D70" s="22" t="n">
+      <c r="D70" s="23" t="n">
         <v>11551251000000</v>
       </c>
       <c r="E70" s="22" t="s">
@@ -5964,7 +5975,7 @@
       <c r="C71" s="22" t="s">
         <v>137</v>
       </c>
-      <c r="D71" s="22" t="n">
+      <c r="D71" s="23" t="n">
         <v>10008995000000</v>
       </c>
       <c r="E71" s="22" t="s">
@@ -5993,7 +6004,7 @@
       <c r="C72" s="22" t="s">
         <v>139</v>
       </c>
-      <c r="D72" s="22" t="n">
+      <c r="D72" s="23" t="n">
         <v>10780123000000</v>
       </c>
       <c r="E72" s="22" t="s">
@@ -6022,7 +6033,7 @@
       <c r="C73" s="22" t="s">
         <v>139</v>
       </c>
-      <c r="D73" s="22" t="n">
+      <c r="D73" s="23" t="n">
         <v>10780123000000</v>
       </c>
       <c r="E73" s="22" t="s">
@@ -6051,7 +6062,7 @@
       <c r="C74" s="22" t="s">
         <v>140</v>
       </c>
-      <c r="D74" s="22" t="n">
+      <c r="D74" s="23" t="n">
         <v>641351000000</v>
       </c>
       <c r="E74" s="22" t="s">
@@ -6101,7 +6112,7 @@
       <c r="C76" s="22" t="s">
         <v>149</v>
       </c>
-      <c r="D76" s="22" t="n">
+      <c r="D76" s="23" t="n">
         <v>73949000000</v>
       </c>
       <c r="E76" s="22" t="s">
@@ -6130,7 +6141,7 @@
       <c r="C77" s="22" t="s">
         <v>152</v>
       </c>
-      <c r="D77" s="22" t="n">
+      <c r="D77" s="23" t="n">
         <v>992964000000</v>
       </c>
       <c r="E77" s="22" t="s">
@@ -6159,7 +6170,7 @@
       <c r="C78" s="22" t="s">
         <v>155</v>
       </c>
-      <c r="D78" s="22" t="n">
+      <c r="D78" s="23" t="n">
         <v>-166008000000</v>
       </c>
       <c r="E78" s="22" t="s">
@@ -6188,7 +6199,7 @@
       <c r="C79" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="D79" s="22" t="n">
+      <c r="D79" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E79" s="22" t="s">
@@ -6217,7 +6228,7 @@
       <c r="C80" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="D80" s="22" t="n">
+      <c r="D80" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E80" s="22" t="s">
@@ -6246,7 +6257,7 @@
       <c r="C81" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="D81" s="22" t="n">
+      <c r="D81" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E81" s="22" t="s">
@@ -6275,7 +6286,7 @@
       <c r="C82" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="D82" s="22" t="n">
+      <c r="D82" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E82" s="22" t="s">
@@ -6304,7 +6315,7 @@
       <c r="C83" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="D83" s="22" t="n">
+      <c r="D83" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E83" s="22" t="s">
@@ -6333,7 +6344,7 @@
       <c r="C84" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="D84" s="22" t="n">
+      <c r="D84" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E84" s="22" t="s">
@@ -6362,7 +6373,7 @@
       <c r="C85" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="D85" s="22" t="n">
+      <c r="D85" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E85" s="22" t="s">
@@ -6391,7 +6402,7 @@
       <c r="C86" s="22" t="s">
         <v>168</v>
       </c>
-      <c r="D86" s="22" t="n">
+      <c r="D86" s="23" t="n">
         <v>529000000</v>
       </c>
       <c r="E86" s="22" t="s">
@@ -6441,7 +6452,7 @@
       <c r="C88" s="22" t="s">
         <v>173</v>
       </c>
-      <c r="D88" s="22" t="n">
+      <c r="D88" s="23" t="n">
         <v>-176000000</v>
       </c>
       <c r="E88" s="22" t="s">
@@ -6470,7 +6481,7 @@
       <c r="C89" s="22" t="s">
         <v>173</v>
       </c>
-      <c r="D89" s="22" t="n">
+      <c r="D89" s="23" t="n">
         <v>-176000000</v>
       </c>
       <c r="E89" s="22" t="s">
@@ -6499,7 +6510,7 @@
       <c r="C90" s="22" t="s">
         <v>173</v>
       </c>
-      <c r="D90" s="22" t="n">
+      <c r="D90" s="23" t="n">
         <v>-176000000</v>
       </c>
       <c r="E90" s="22" t="s">
@@ -6528,7 +6539,7 @@
       <c r="C91" s="22" t="s">
         <v>173</v>
       </c>
-      <c r="D91" s="22" t="n">
+      <c r="D91" s="23" t="n">
         <v>-176000000</v>
       </c>
       <c r="E91" s="22" t="s">
@@ -6557,7 +6568,7 @@
       <c r="C92" s="22" t="s">
         <v>173</v>
       </c>
-      <c r="D92" s="22" t="n">
+      <c r="D92" s="23" t="n">
         <v>-176000000</v>
       </c>
       <c r="E92" s="22" t="s">
@@ -6586,7 +6597,7 @@
       <c r="C93" s="22" t="s">
         <v>173</v>
       </c>
-      <c r="D93" s="22" t="n">
+      <c r="D93" s="23" t="n">
         <v>-176000000</v>
       </c>
       <c r="E93" s="22" t="s">
@@ -6615,7 +6626,7 @@
       <c r="C94" s="22" t="s">
         <v>173</v>
       </c>
-      <c r="D94" s="22" t="n">
+      <c r="D94" s="23" t="n">
         <v>-176000000</v>
       </c>
       <c r="E94" s="22" t="s">
@@ -6644,7 +6655,7 @@
       <c r="C95" s="22" t="s">
         <v>188</v>
       </c>
-      <c r="D95" s="22" t="n">
+      <c r="D95" s="23" t="n">
         <v>15485000000</v>
       </c>
       <c r="E95" s="22" t="s">
@@ -6781,7 +6792,7 @@
       <c r="C100" s="22" t="s">
         <v>194</v>
       </c>
-      <c r="D100" s="22" t="n">
+      <c r="D100" s="23" t="n">
         <v>1207000000</v>
       </c>
       <c r="E100" s="22" t="s">
@@ -6810,7 +6821,7 @@
       <c r="C101" s="22" t="s">
         <v>196</v>
       </c>
-      <c r="D101" s="22" t="n">
+      <c r="D101" s="23" t="n">
         <v>615000000</v>
       </c>
       <c r="E101" s="22" t="s">
@@ -6839,7 +6850,7 @@
       <c r="C102" s="22" t="s">
         <v>198</v>
       </c>
-      <c r="D102" s="22" t="n">
+      <c r="D102" s="23" t="n">
         <v>1603000000</v>
       </c>
       <c r="E102" s="22" t="s">
@@ -6868,7 +6879,7 @@
       <c r="C103" s="22" t="s">
         <v>200</v>
       </c>
-      <c r="D103" s="22" t="n">
+      <c r="D103" s="23" t="n">
         <v>1273000000</v>
       </c>
       <c r="E103" s="22" t="s">
@@ -6918,7 +6929,7 @@
       <c r="C105" s="22" t="s">
         <v>204</v>
       </c>
-      <c r="D105" s="22" t="n">
+      <c r="D105" s="23" t="n">
         <v>224000000</v>
       </c>
       <c r="E105" s="22" t="s">
@@ -6947,7 +6958,7 @@
       <c r="C106" s="22" t="s">
         <v>206</v>
       </c>
-      <c r="D106" s="22" t="n">
+      <c r="D106" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E106" s="22" t="s">
@@ -6976,7 +6987,7 @@
       <c r="C107" s="22" t="s">
         <v>206</v>
       </c>
-      <c r="D107" s="22" t="n">
+      <c r="D107" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E107" s="22" t="s">
@@ -7005,7 +7016,7 @@
       <c r="C108" s="22" t="s">
         <v>206</v>
       </c>
-      <c r="D108" s="22" t="n">
+      <c r="D108" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E108" s="22" t="s">
@@ -7034,7 +7045,7 @@
       <c r="C109" s="22" t="s">
         <v>206</v>
       </c>
-      <c r="D109" s="22" t="n">
+      <c r="D109" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E109" s="22" t="s">
@@ -7063,7 +7074,7 @@
       <c r="C110" s="22" t="s">
         <v>206</v>
       </c>
-      <c r="D110" s="22" t="n">
+      <c r="D110" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E110" s="22" t="s">
@@ -7092,7 +7103,7 @@
       <c r="C111" s="22" t="s">
         <v>206</v>
       </c>
-      <c r="D111" s="22" t="n">
+      <c r="D111" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E111" s="22" t="s">
@@ -7121,7 +7132,7 @@
       <c r="C112" s="22" t="s">
         <v>206</v>
       </c>
-      <c r="D112" s="22" t="n">
+      <c r="D112" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E112" s="22" t="s">
@@ -7150,7 +7161,7 @@
       <c r="C113" s="22" t="s">
         <v>210</v>
       </c>
-      <c r="D113" s="22" t="n">
+      <c r="D113" s="23" t="n">
         <v>20407000000</v>
       </c>
       <c r="E113" s="22" t="s">
@@ -7179,7 +7190,7 @@
       <c r="C114" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="D114" s="22" t="n">
+      <c r="D114" s="23" t="n">
         <v>7574000000</v>
       </c>
       <c r="E114" s="22" t="s">
@@ -7208,7 +7219,7 @@
       <c r="C115" s="22" t="s">
         <v>212</v>
       </c>
-      <c r="D115" s="22" t="n">
+      <c r="D115" s="23" t="n">
         <v>538000000</v>
       </c>
       <c r="E115" s="22" t="s">
@@ -7237,7 +7248,7 @@
       <c r="C116" s="22" t="s">
         <v>214</v>
       </c>
-      <c r="D116" s="22" t="n">
+      <c r="D116" s="23" t="n">
         <v>0.214948764315853</v>
       </c>
       <c r="E116" s="22" t="s">
@@ -7266,7 +7277,7 @@
       <c r="C117" s="22" t="s">
         <v>214</v>
       </c>
-      <c r="D117" s="22" t="n">
+      <c r="D117" s="23" t="n">
         <v>0.214948764315853</v>
       </c>
       <c r="E117" s="22" t="s">
@@ -7295,7 +7306,7 @@
       <c r="C118" s="22" t="s">
         <v>217</v>
       </c>
-      <c r="D118" s="22" t="n">
+      <c r="D118" s="23" t="n">
         <v>255000000</v>
       </c>
       <c r="E118" s="22" t="s">
@@ -7324,7 +7335,7 @@
       <c r="C119" s="22" t="s">
         <v>220</v>
       </c>
-      <c r="D119" s="22" t="n">
+      <c r="D119" s="23" t="n">
         <v>12762000000</v>
       </c>
       <c r="E119" s="22" t="s">
@@ -7407,7 +7418,7 @@
       <c r="C122" s="22" t="s">
         <v>225</v>
       </c>
-      <c r="D122" s="22" t="n">
+      <c r="D122" s="23" t="n">
         <v>12314000000</v>
       </c>
       <c r="E122" s="22" t="s">
@@ -7436,7 +7447,7 @@
       <c r="C123" s="22" t="s">
         <v>225</v>
       </c>
-      <c r="D123" s="22" t="n">
+      <c r="D123" s="23" t="n">
         <v>12314000000</v>
       </c>
       <c r="E123" s="22" t="s">
@@ -7465,7 +7476,7 @@
       <c r="C124" s="22" t="s">
         <v>225</v>
       </c>
-      <c r="D124" s="22" t="n">
+      <c r="D124" s="23" t="n">
         <v>12314000000</v>
       </c>
       <c r="E124" s="22" t="s">
@@ -7494,7 +7505,7 @@
       <c r="C125" s="22" t="s">
         <v>227</v>
       </c>
-      <c r="D125" s="22" t="n">
+      <c r="D125" s="23" t="n">
         <v>-176000000</v>
       </c>
       <c r="E125" s="22" t="s">
@@ -7523,7 +7534,7 @@
       <c r="C126" s="22" t="s">
         <v>227</v>
       </c>
-      <c r="D126" s="22" t="n">
+      <c r="D126" s="23" t="n">
         <v>-176000000</v>
       </c>
       <c r="E126" s="22" t="s">
@@ -7552,7 +7563,7 @@
       <c r="C127" s="22" t="s">
         <v>227</v>
       </c>
-      <c r="D127" s="22" t="n">
+      <c r="D127" s="23" t="n">
         <v>-176000000</v>
       </c>
       <c r="E127" s="22" t="s">
@@ -7581,7 +7592,7 @@
       <c r="C128" s="22" t="s">
         <v>227</v>
       </c>
-      <c r="D128" s="22" t="n">
+      <c r="D128" s="23" t="n">
         <v>-176000000</v>
       </c>
       <c r="E128" s="22" t="s">
@@ -7610,7 +7621,7 @@
       <c r="C129" s="22" t="s">
         <v>227</v>
       </c>
-      <c r="D129" s="22" t="n">
+      <c r="D129" s="23" t="n">
         <v>-176000000</v>
       </c>
       <c r="E129" s="22" t="s">
@@ -7639,7 +7650,7 @@
       <c r="C130" s="22" t="s">
         <v>227</v>
       </c>
-      <c r="D130" s="22" t="n">
+      <c r="D130" s="23" t="n">
         <v>-176000000</v>
       </c>
       <c r="E130" s="22" t="s">
@@ -7668,7 +7679,7 @@
       <c r="C131" s="22" t="s">
         <v>227</v>
       </c>
-      <c r="D131" s="22" t="n">
+      <c r="D131" s="23" t="n">
         <v>-176000000</v>
       </c>
       <c r="E131" s="22" t="s">
@@ -7697,7 +7708,7 @@
       <c r="C132" s="22" t="s">
         <v>228</v>
       </c>
-      <c r="D132" s="22" t="n">
+      <c r="D132" s="23" t="n">
         <v>529000000</v>
       </c>
       <c r="E132" s="22" t="s">
@@ -7747,7 +7758,7 @@
       <c r="C134" s="22" t="s">
         <v>230</v>
       </c>
-      <c r="D134" s="22" t="n">
+      <c r="D134" s="23" t="n">
         <v>169000000</v>
       </c>
       <c r="E134" s="22" t="s">
@@ -7803,7 +7814,7 @@
       <c r="C136" s="22" t="s">
         <v>235</v>
       </c>
-      <c r="D136" s="22" t="n">
+      <c r="D136" s="23" t="n">
         <v>151615085</v>
       </c>
       <c r="E136" s="22" t="s">
@@ -7832,7 +7843,7 @@
       <c r="C137" s="22" t="s">
         <v>131</v>
       </c>
-      <c r="D137" s="22" t="n">
+      <c r="D137" s="23" t="n">
         <v>14041518000000</v>
       </c>
       <c r="E137" s="22" t="s">
@@ -7861,7 +7872,7 @@
       <c r="C138" s="22" t="s">
         <v>137</v>
       </c>
-      <c r="D138" s="22" t="n">
+      <c r="D138" s="23" t="n">
         <v>11551251000000</v>
       </c>
       <c r="E138" s="22" t="s">
@@ -7890,7 +7901,7 @@
       <c r="C139" s="22" t="s">
         <v>139</v>
       </c>
-      <c r="D139" s="22" t="n">
+      <c r="D139" s="23" t="n">
         <v>12796384500000</v>
       </c>
       <c r="E139" s="22" t="s">
@@ -7919,7 +7930,7 @@
       <c r="C140" s="22" t="s">
         <v>139</v>
       </c>
-      <c r="D140" s="22" t="n">
+      <c r="D140" s="23" t="n">
         <v>12796384500000</v>
       </c>
       <c r="E140" s="22" t="s">
@@ -7948,7 +7959,7 @@
       <c r="C141" s="22" t="s">
         <v>140</v>
       </c>
-      <c r="D141" s="22" t="n">
+      <c r="D141" s="23" t="n">
         <v>698261000000</v>
       </c>
       <c r="E141" s="22" t="s">
@@ -7977,7 +7988,7 @@
       <c r="C142" s="22" t="s">
         <v>146</v>
       </c>
-      <c r="D142" s="22" t="n">
+      <c r="D142" s="23" t="n">
         <v>-33125000000</v>
       </c>
       <c r="E142" s="22" t="s">
@@ -8006,7 +8017,7 @@
       <c r="C143" s="22" t="s">
         <v>149</v>
       </c>
-      <c r="D143" s="22" t="n">
+      <c r="D143" s="23" t="n">
         <v>120961000000</v>
       </c>
       <c r="E143" s="22" t="s">
@@ -8035,7 +8046,7 @@
       <c r="C144" s="22" t="s">
         <v>152</v>
       </c>
-      <c r="D144" s="22" t="n">
+      <c r="D144" s="23" t="n">
         <v>1483629000000</v>
       </c>
       <c r="E144" s="22" t="s">
@@ -8064,7 +8075,7 @@
       <c r="C145" s="22" t="s">
         <v>155</v>
       </c>
-      <c r="D145" s="22" t="n">
+      <c r="D145" s="23" t="n">
         <v>220541000000</v>
       </c>
       <c r="E145" s="22" t="s">
@@ -8093,7 +8104,7 @@
       <c r="C146" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="D146" s="22" t="n">
+      <c r="D146" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E146" s="22" t="s">
@@ -8122,7 +8133,7 @@
       <c r="C147" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="D147" s="22" t="n">
+      <c r="D147" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E147" s="22" t="s">
@@ -8151,7 +8162,7 @@
       <c r="C148" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="D148" s="22" t="n">
+      <c r="D148" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E148" s="22" t="s">
@@ -8180,7 +8191,7 @@
       <c r="C149" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="D149" s="22" t="n">
+      <c r="D149" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E149" s="22" t="s">
@@ -8209,7 +8220,7 @@
       <c r="C150" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="D150" s="22" t="n">
+      <c r="D150" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E150" s="22" t="s">
@@ -8238,7 +8249,7 @@
       <c r="C151" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="D151" s="22" t="n">
+      <c r="D151" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E151" s="22" t="s">
@@ -8267,7 +8278,7 @@
       <c r="C152" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="D152" s="22" t="n">
+      <c r="D152" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E152" s="22" t="s">
@@ -8296,7 +8307,7 @@
       <c r="C153" s="22" t="s">
         <v>158</v>
       </c>
-      <c r="D153" s="22" t="n">
+      <c r="D153" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E153" s="22" t="s">
@@ -8325,7 +8336,7 @@
       <c r="C154" s="22" t="s">
         <v>168</v>
       </c>
-      <c r="D154" s="22" t="n">
+      <c r="D154" s="23" t="n">
         <v>1126000000</v>
       </c>
       <c r="E154" s="22" t="s">
@@ -8375,7 +8386,7 @@
       <c r="C156" s="22" t="s">
         <v>173</v>
       </c>
-      <c r="D156" s="22" t="n">
+      <c r="D156" s="23" t="n">
         <v>189000000</v>
       </c>
       <c r="E156" s="22" t="s">
@@ -8404,7 +8415,7 @@
       <c r="C157" s="22" t="s">
         <v>173</v>
       </c>
-      <c r="D157" s="22" t="n">
+      <c r="D157" s="23" t="n">
         <v>189000000</v>
       </c>
       <c r="E157" s="22" t="s">
@@ -8433,7 +8444,7 @@
       <c r="C158" s="22" t="s">
         <v>173</v>
       </c>
-      <c r="D158" s="22" t="n">
+      <c r="D158" s="23" t="n">
         <v>189000000</v>
       </c>
       <c r="E158" s="22" t="s">
@@ -8462,7 +8473,7 @@
       <c r="C159" s="22" t="s">
         <v>173</v>
       </c>
-      <c r="D159" s="22" t="n">
+      <c r="D159" s="23" t="n">
         <v>189000000</v>
       </c>
       <c r="E159" s="22" t="s">
@@ -8491,7 +8502,7 @@
       <c r="C160" s="22" t="s">
         <v>173</v>
       </c>
-      <c r="D160" s="22" t="n">
+      <c r="D160" s="23" t="n">
         <v>189000000</v>
       </c>
       <c r="E160" s="22" t="s">
@@ -8520,7 +8531,7 @@
       <c r="C161" s="22" t="s">
         <v>173</v>
       </c>
-      <c r="D161" s="22" t="n">
+      <c r="D161" s="23" t="n">
         <v>189000000</v>
       </c>
       <c r="E161" s="22" t="s">
@@ -8549,7 +8560,7 @@
       <c r="C162" s="22" t="s">
         <v>173</v>
       </c>
-      <c r="D162" s="22" t="n">
+      <c r="D162" s="23" t="n">
         <v>189000000</v>
       </c>
       <c r="E162" s="22" t="s">
@@ -8578,7 +8589,7 @@
       <c r="C163" s="22" t="s">
         <v>188</v>
       </c>
-      <c r="D163" s="22" t="n">
+      <c r="D163" s="23" t="n">
         <v>18474000000</v>
       </c>
       <c r="E163" s="22" t="s">
@@ -8715,7 +8726,7 @@
       <c r="C168" s="22" t="s">
         <v>194</v>
       </c>
-      <c r="D168" s="22" t="n">
+      <c r="D168" s="23" t="n">
         <v>1424000000</v>
       </c>
       <c r="E168" s="22" t="s">
@@ -8744,7 +8755,7 @@
       <c r="C169" s="22" t="s">
         <v>196</v>
       </c>
-      <c r="D169" s="22" t="n">
+      <c r="D169" s="23" t="n">
         <v>705000000</v>
       </c>
       <c r="E169" s="22" t="s">
@@ -8773,7 +8784,7 @@
       <c r="C170" s="22" t="s">
         <v>198</v>
       </c>
-      <c r="D170" s="22" t="n">
+      <c r="D170" s="23" t="n">
         <v>1981000000</v>
       </c>
       <c r="E170" s="22" t="s">
@@ -8802,7 +8813,7 @@
       <c r="C171" s="22" t="s">
         <v>200</v>
       </c>
-      <c r="D171" s="22" t="n">
+      <c r="D171" s="23" t="n">
         <v>1355000000</v>
       </c>
       <c r="E171" s="22" t="s">
@@ -8852,7 +8863,7 @@
       <c r="C173" s="22" t="s">
         <v>204</v>
       </c>
-      <c r="D173" s="22" t="n">
+      <c r="D173" s="23" t="n">
         <v>277000000</v>
       </c>
       <c r="E173" s="22" t="s">
@@ -8881,7 +8892,7 @@
       <c r="C174" s="22" t="s">
         <v>206</v>
       </c>
-      <c r="D174" s="22" t="n">
+      <c r="D174" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E174" s="22" t="s">
@@ -8910,7 +8921,7 @@
       <c r="C175" s="22" t="s">
         <v>206</v>
       </c>
-      <c r="D175" s="22" t="n">
+      <c r="D175" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E175" s="22" t="s">
@@ -8939,7 +8950,7 @@
       <c r="C176" s="22" t="s">
         <v>206</v>
       </c>
-      <c r="D176" s="22" t="n">
+      <c r="D176" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E176" s="22" t="s">
@@ -8968,7 +8979,7 @@
       <c r="C177" s="22" t="s">
         <v>206</v>
       </c>
-      <c r="D177" s="22" t="n">
+      <c r="D177" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E177" s="22" t="s">
@@ -8997,7 +9008,7 @@
       <c r="C178" s="22" t="s">
         <v>206</v>
       </c>
-      <c r="D178" s="22" t="n">
+      <c r="D178" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E178" s="22" t="s">
@@ -9026,7 +9037,7 @@
       <c r="C179" s="22" t="s">
         <v>206</v>
       </c>
-      <c r="D179" s="22" t="n">
+      <c r="D179" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E179" s="22" t="s">
@@ -9055,7 +9066,7 @@
       <c r="C180" s="22" t="s">
         <v>206</v>
       </c>
-      <c r="D180" s="22" t="n">
+      <c r="D180" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E180" s="22" t="s">
@@ -9084,7 +9095,7 @@
       <c r="C181" s="22" t="s">
         <v>210</v>
       </c>
-      <c r="D181" s="22" t="n">
+      <c r="D181" s="23" t="n">
         <v>24216000000</v>
       </c>
       <c r="E181" s="22" t="s">
@@ -9113,7 +9124,7 @@
       <c r="C182" s="22" t="s">
         <v>77</v>
       </c>
-      <c r="D182" s="22" t="n">
+      <c r="D182" s="23" t="n">
         <v>7045000000</v>
       </c>
       <c r="E182" s="22" t="s">
@@ -9142,7 +9153,7 @@
       <c r="C183" s="22" t="s">
         <v>212</v>
       </c>
-      <c r="D183" s="22" t="n">
+      <c r="D183" s="23" t="n">
         <v>614000000</v>
       </c>
       <c r="E183" s="22" t="s">
@@ -9171,7 +9182,7 @@
       <c r="C184" s="22" t="s">
         <v>214</v>
       </c>
-      <c r="D184" s="22" t="n">
+      <c r="D184" s="23" t="n">
         <v>0.220107625672661</v>
       </c>
       <c r="E184" s="22" t="s">
@@ -9200,7 +9211,7 @@
       <c r="C185" s="22" t="s">
         <v>214</v>
       </c>
-      <c r="D185" s="22" t="n">
+      <c r="D185" s="23" t="n">
         <v>0.220107625672661</v>
       </c>
       <c r="E185" s="22" t="s">
@@ -9229,7 +9240,7 @@
       <c r="C186" s="22" t="s">
         <v>217</v>
       </c>
-      <c r="D186" s="22" t="n">
+      <c r="D186" s="23" t="n">
         <v>375000000</v>
       </c>
       <c r="E186" s="22" t="s">
@@ -9258,7 +9269,7 @@
       <c r="C187" s="22" t="s">
         <v>220</v>
       </c>
-      <c r="D187" s="22" t="n">
+      <c r="D187" s="23" t="n">
         <v>11468000000</v>
       </c>
       <c r="E187" s="22" t="s">
@@ -9341,7 +9352,7 @@
       <c r="C190" s="22" t="s">
         <v>225</v>
       </c>
-      <c r="D190" s="22" t="n">
+      <c r="D190" s="23" t="n">
         <v>12768000000</v>
       </c>
       <c r="E190" s="22" t="s">
@@ -9370,7 +9381,7 @@
       <c r="C191" s="22" t="s">
         <v>225</v>
       </c>
-      <c r="D191" s="22" t="n">
+      <c r="D191" s="23" t="n">
         <v>12768000000</v>
       </c>
       <c r="E191" s="22" t="s">
@@ -9399,7 +9410,7 @@
       <c r="C192" s="22" t="s">
         <v>225</v>
       </c>
-      <c r="D192" s="22" t="n">
+      <c r="D192" s="23" t="n">
         <v>12768000000</v>
       </c>
       <c r="E192" s="22" t="s">
@@ -9428,7 +9439,7 @@
       <c r="C193" s="22" t="s">
         <v>227</v>
       </c>
-      <c r="D193" s="22" t="n">
+      <c r="D193" s="23" t="n">
         <v>189000000</v>
       </c>
       <c r="E193" s="22" t="s">
@@ -9457,7 +9468,7 @@
       <c r="C194" s="22" t="s">
         <v>227</v>
       </c>
-      <c r="D194" s="22" t="n">
+      <c r="D194" s="23" t="n">
         <v>189000000</v>
       </c>
       <c r="E194" s="22" t="s">
@@ -9486,7 +9497,7 @@
       <c r="C195" s="22" t="s">
         <v>227</v>
       </c>
-      <c r="D195" s="22" t="n">
+      <c r="D195" s="23" t="n">
         <v>189000000</v>
       </c>
       <c r="E195" s="22" t="s">
@@ -9515,7 +9526,7 @@
       <c r="C196" s="22" t="s">
         <v>227</v>
       </c>
-      <c r="D196" s="22" t="n">
+      <c r="D196" s="23" t="n">
         <v>189000000</v>
       </c>
       <c r="E196" s="22" t="s">
@@ -9544,7 +9555,7 @@
       <c r="C197" s="22" t="s">
         <v>227</v>
       </c>
-      <c r="D197" s="22" t="n">
+      <c r="D197" s="23" t="n">
         <v>189000000</v>
       </c>
       <c r="E197" s="22" t="s">
@@ -9573,7 +9584,7 @@
       <c r="C198" s="22" t="s">
         <v>227</v>
       </c>
-      <c r="D198" s="22" t="n">
+      <c r="D198" s="23" t="n">
         <v>189000000</v>
       </c>
       <c r="E198" s="22" t="s">
@@ -9602,7 +9613,7 @@
       <c r="C199" s="22" t="s">
         <v>227</v>
       </c>
-      <c r="D199" s="22" t="n">
+      <c r="D199" s="23" t="n">
         <v>189000000</v>
       </c>
       <c r="E199" s="22" t="s">
@@ -9631,7 +9642,7 @@
       <c r="C200" s="22" t="s">
         <v>228</v>
       </c>
-      <c r="D200" s="22" t="n">
+      <c r="D200" s="23" t="n">
         <v>1126000000</v>
       </c>
       <c r="E200" s="22" t="s">
@@ -9681,7 +9692,7 @@
       <c r="C202" s="22" t="s">
         <v>230</v>
       </c>
-      <c r="D202" s="22" t="n">
+      <c r="D202" s="23" t="n">
         <v>227000000</v>
       </c>
       <c r="E202" s="22" t="s">
@@ -9737,7 +9748,7 @@
       <c r="C204" s="22" t="s">
         <v>235</v>
       </c>
-      <c r="D204" s="22" t="n">
+      <c r="D204" s="23" t="n">
         <v>160866521</v>
       </c>
       <c r="E204" s="22" t="s">
@@ -9768,17 +9779,17 @@
       <c r="I205" s="22"/>
     </row>
     <row r="206" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A206" s="23" t="s">
+      <c r="A206" s="24" t="s">
         <v>253</v>
       </c>
-      <c r="B206" s="23"/>
-      <c r="C206" s="23"/>
-      <c r="D206" s="23"/>
-      <c r="E206" s="23"/>
-      <c r="F206" s="23"/>
-      <c r="G206" s="23"/>
-      <c r="H206" s="23"/>
-      <c r="I206" s="23"/>
+      <c r="B206" s="24"/>
+      <c r="C206" s="24"/>
+      <c r="D206" s="24"/>
+      <c r="E206" s="24"/>
+      <c r="F206" s="24"/>
+      <c r="G206" s="24"/>
+      <c r="H206" s="24"/>
+      <c r="I206" s="24"/>
     </row>
     <row r="207" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A207" s="22" t="s">
@@ -9788,7 +9799,7 @@
       <c r="C207" s="22" t="s">
         <v>255</v>
       </c>
-      <c r="D207" s="22" t="n">
+      <c r="D207" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E207" s="22"/>
@@ -9807,7 +9818,7 @@
       <c r="C208" s="22" t="s">
         <v>257</v>
       </c>
-      <c r="D208" s="22" t="n">
+      <c r="D208" s="23" t="n">
         <v>0.0527057133023256</v>
       </c>
       <c r="E208" s="22"/>
@@ -9826,7 +9837,7 @@
       <c r="C209" s="22" t="s">
         <v>259</v>
       </c>
-      <c r="D209" s="22" t="n">
+      <c r="D209" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E209" s="22"/>
@@ -9845,7 +9856,7 @@
       <c r="C210" s="22" t="s">
         <v>261</v>
       </c>
-      <c r="D210" s="22" t="n">
+      <c r="D210" s="23" t="n">
         <v>0.00603774529497898</v>
       </c>
       <c r="E210" s="22"/>
@@ -9883,7 +9894,7 @@
       <c r="C212" s="22" t="s">
         <v>265</v>
       </c>
-      <c r="D212" s="22" t="n">
+      <c r="D212" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E212" s="22"/>
@@ -9940,7 +9951,7 @@
       <c r="C215" s="22" t="s">
         <v>271</v>
       </c>
-      <c r="D215" s="22" t="n">
+      <c r="D215" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E215" s="22"/>
@@ -9978,7 +9989,7 @@
       <c r="C217" s="22" t="s">
         <v>275</v>
       </c>
-      <c r="D217" s="22" t="n">
+      <c r="D217" s="23" t="n">
         <v>1981000000</v>
       </c>
       <c r="E217" s="22"/>
@@ -9997,7 +10008,7 @@
       <c r="C218" s="22" t="s">
         <v>277</v>
       </c>
-      <c r="D218" s="22" t="n">
+      <c r="D218" s="23" t="n">
         <v>0.157634569861644</v>
       </c>
       <c r="E218" s="22"/>
@@ -10035,7 +10046,7 @@
       <c r="C220" s="22" t="s">
         <v>281</v>
       </c>
-      <c r="D220" s="22" t="n">
+      <c r="D220" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E220" s="22"/>
@@ -10054,7 +10065,7 @@
       <c r="C221" s="22" t="s">
         <v>283</v>
       </c>
-      <c r="D221" s="22" t="n">
+      <c r="D221" s="23" t="n">
         <v>0.322706087151842</v>
       </c>
       <c r="E221" s="22"/>
@@ -10073,7 +10084,7 @@
       <c r="C222" s="22" t="s">
         <v>285</v>
       </c>
-      <c r="D222" s="22" t="n">
+      <c r="D222" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E222" s="22"/>
@@ -10092,7 +10103,7 @@
       <c r="C223" s="22" t="s">
         <v>287</v>
       </c>
-      <c r="D223" s="22" t="n">
+      <c r="D223" s="23" t="n">
         <v>0.351363458200347</v>
       </c>
       <c r="E223" s="22"/>
@@ -10111,7 +10122,7 @@
       <c r="C224" s="22" t="s">
         <v>289</v>
       </c>
-      <c r="D224" s="22" t="n">
+      <c r="D224" s="23" t="n">
         <v>0.214948764315853</v>
       </c>
       <c r="E224" s="22"/>
@@ -10130,7 +10141,7 @@
       <c r="C225" s="22" t="s">
         <v>291</v>
       </c>
-      <c r="D225" s="22" t="n">
+      <c r="D225" s="23" t="n">
         <v>0.0259224775812221</v>
       </c>
       <c r="E225" s="22"/>
@@ -10149,7 +10160,7 @@
       <c r="C226" s="22" t="s">
         <v>293</v>
       </c>
-      <c r="D226" s="22" t="n">
+      <c r="D226" s="23" t="n">
         <v>0</v>
       </c>
       <c r="E226" s="22"/>
@@ -10168,7 +10179,7 @@
       <c r="C227" s="22" t="s">
         <v>295</v>
       </c>
-      <c r="D227" s="22" t="n">
+      <c r="D227" s="23" t="n">
         <v>0.0154856293359762</v>
       </c>
       <c r="E227" s="22"/>
@@ -10187,7 +10198,7 @@
       <c r="C228" s="22" t="s">
         <v>297</v>
       </c>
-      <c r="D228" s="22" t="n">
+      <c r="D228" s="23" t="n">
         <v>0.00780475718533201</v>
       </c>
       <c r="E228" s="22"/>
@@ -10206,7 +10217,7 @@
       <c r="C229" s="22" t="s">
         <v>299</v>
       </c>
-      <c r="D229" s="22" t="n">
+      <c r="D229" s="23" t="n">
         <v>0.0489594131249502</v>
       </c>
       <c r="E229" s="22"/>
@@ -10225,7 +10236,7 @@
       <c r="C230" s="22" t="s">
         <v>301</v>
       </c>
-      <c r="D230" s="22" t="n">
+      <c r="D230" s="23" t="n">
         <v>0.163312185321282</v>
       </c>
       <c r="E230" s="22"/>
@@ -10244,7 +10255,7 @@
       <c r="C231" s="22" t="s">
         <v>303</v>
       </c>
-      <c r="D231" s="22" t="n">
+      <c r="D231" s="23" t="n">
         <v>0.025</v>
       </c>
       <c r="E231" s="22"/>
@@ -10256,171 +10267,201 @@
       </c>
     </row>
     <row r="232" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A232" s="23" t="s">
+      <c r="A232" s="24" t="s">
         <v>305</v>
       </c>
-      <c r="B232" s="23"/>
-      <c r="C232" s="23"/>
-      <c r="D232" s="23"/>
-      <c r="E232" s="23"/>
-      <c r="F232" s="23"/>
-      <c r="G232" s="23"/>
-      <c r="H232" s="23"/>
-      <c r="I232" s="23"/>
+      <c r="B232" s="24"/>
+      <c r="C232" s="24"/>
+      <c r="D232" s="24"/>
+      <c r="E232" s="24"/>
+      <c r="F232" s="24"/>
+      <c r="G232" s="24"/>
+      <c r="H232" s="24"/>
+      <c r="I232" s="24"/>
     </row>
     <row r="233" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A233" s="22" t="s">
         <v>306</v>
       </c>
       <c r="B233" s="22"/>
-      <c r="C233" s="24" t="s">
+      <c r="C233" s="25" t="s">
         <v>307</v>
       </c>
-      <c r="D233" s="24"/>
-      <c r="E233" s="24"/>
-      <c r="F233" s="24"/>
-      <c r="G233" s="24"/>
-      <c r="H233" s="24"/>
-      <c r="I233" s="24"/>
+      <c r="D233" s="25"/>
+      <c r="E233" s="25"/>
+      <c r="F233" s="25"/>
+      <c r="G233" s="25"/>
+      <c r="H233" s="25"/>
+      <c r="I233" s="25"/>
     </row>
     <row r="234" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A234" s="22" t="s">
         <v>306</v>
       </c>
       <c r="B234" s="22"/>
-      <c r="C234" s="24" t="s">
+      <c r="C234" s="25" t="s">
         <v>308</v>
       </c>
-      <c r="D234" s="24"/>
-      <c r="E234" s="24"/>
-      <c r="F234" s="24"/>
-      <c r="G234" s="24"/>
-      <c r="H234" s="24"/>
-      <c r="I234" s="24"/>
+      <c r="D234" s="25"/>
+      <c r="E234" s="25"/>
+      <c r="F234" s="25"/>
+      <c r="G234" s="25"/>
+      <c r="H234" s="25"/>
+      <c r="I234" s="25"/>
     </row>
     <row r="235" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A235" s="22" t="s">
         <v>306</v>
       </c>
       <c r="B235" s="22"/>
-      <c r="C235" s="24" t="s">
+      <c r="C235" s="25" t="s">
         <v>309</v>
       </c>
-      <c r="D235" s="24"/>
-      <c r="E235" s="24"/>
-      <c r="F235" s="24"/>
-      <c r="G235" s="24"/>
-      <c r="H235" s="24"/>
-      <c r="I235" s="24"/>
+      <c r="D235" s="25"/>
+      <c r="E235" s="25"/>
+      <c r="F235" s="25"/>
+      <c r="G235" s="25"/>
+      <c r="H235" s="25"/>
+      <c r="I235" s="25"/>
     </row>
     <row r="236" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A236" s="22" t="s">
         <v>306</v>
       </c>
       <c r="B236" s="22"/>
-      <c r="C236" s="24" t="s">
+      <c r="C236" s="25" t="s">
         <v>310</v>
       </c>
-      <c r="D236" s="24"/>
-      <c r="E236" s="24"/>
-      <c r="F236" s="24"/>
-      <c r="G236" s="24"/>
-      <c r="H236" s="24"/>
-      <c r="I236" s="24"/>
+      <c r="D236" s="25"/>
+      <c r="E236" s="25"/>
+      <c r="F236" s="25"/>
+      <c r="G236" s="25"/>
+      <c r="H236" s="25"/>
+      <c r="I236" s="25"/>
     </row>
     <row r="237" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A237" s="22" t="s">
         <v>306</v>
       </c>
       <c r="B237" s="22"/>
-      <c r="C237" s="24" t="s">
+      <c r="C237" s="25" t="s">
         <v>311</v>
       </c>
-      <c r="D237" s="24"/>
-      <c r="E237" s="24"/>
-      <c r="F237" s="24"/>
-      <c r="G237" s="24"/>
-      <c r="H237" s="24"/>
-      <c r="I237" s="24"/>
+      <c r="D237" s="25"/>
+      <c r="E237" s="25"/>
+      <c r="F237" s="25"/>
+      <c r="G237" s="25"/>
+      <c r="H237" s="25"/>
+      <c r="I237" s="25"/>
     </row>
     <row r="238" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A238" s="22" t="s">
         <v>306</v>
       </c>
       <c r="B238" s="22"/>
-      <c r="C238" s="24" t="s">
+      <c r="C238" s="25" t="s">
         <v>312</v>
       </c>
-      <c r="D238" s="24"/>
-      <c r="E238" s="24"/>
-      <c r="F238" s="24"/>
-      <c r="G238" s="24"/>
-      <c r="H238" s="24"/>
-      <c r="I238" s="24"/>
+      <c r="D238" s="25"/>
+      <c r="E238" s="25"/>
+      <c r="F238" s="25"/>
+      <c r="G238" s="25"/>
+      <c r="H238" s="25"/>
+      <c r="I238" s="25"/>
     </row>
     <row r="239" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A239" s="22" t="s">
         <v>306</v>
       </c>
       <c r="B239" s="22"/>
-      <c r="C239" s="24" t="s">
+      <c r="C239" s="25" t="s">
         <v>313</v>
       </c>
-      <c r="D239" s="24"/>
-      <c r="E239" s="24"/>
-      <c r="F239" s="24"/>
-      <c r="G239" s="24"/>
-      <c r="H239" s="24"/>
-      <c r="I239" s="24"/>
+      <c r="D239" s="25"/>
+      <c r="E239" s="25"/>
+      <c r="F239" s="25"/>
+      <c r="G239" s="25"/>
+      <c r="H239" s="25"/>
+      <c r="I239" s="25"/>
     </row>
     <row r="240" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A240" s="22" t="s">
         <v>306</v>
       </c>
       <c r="B240" s="22"/>
-      <c r="C240" s="24" t="s">
+      <c r="C240" s="25" t="s">
         <v>314</v>
       </c>
-      <c r="D240" s="24"/>
-      <c r="E240" s="24"/>
-      <c r="F240" s="24"/>
-      <c r="G240" s="24"/>
-      <c r="H240" s="24"/>
-      <c r="I240" s="24"/>
+      <c r="D240" s="25"/>
+      <c r="E240" s="25"/>
+      <c r="F240" s="25"/>
+      <c r="G240" s="25"/>
+      <c r="H240" s="25"/>
+      <c r="I240" s="25"/>
     </row>
     <row r="241" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A241" s="22" t="s">
         <v>306</v>
       </c>
       <c r="B241" s="22"/>
-      <c r="C241" s="24" t="s">
+      <c r="C241" s="25" t="s">
         <v>315</v>
       </c>
-      <c r="D241" s="24"/>
-      <c r="E241" s="24"/>
-      <c r="F241" s="24"/>
-      <c r="G241" s="24"/>
-      <c r="H241" s="24"/>
-      <c r="I241" s="24"/>
+      <c r="D241" s="25"/>
+      <c r="E241" s="25"/>
+      <c r="F241" s="25"/>
+      <c r="G241" s="25"/>
+      <c r="H241" s="25"/>
+      <c r="I241" s="25"/>
     </row>
     <row r="242" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A242" s="22" t="s">
         <v>306</v>
       </c>
       <c r="B242" s="22"/>
-      <c r="C242" s="24" t="s">
+      <c r="C242" s="25" t="s">
         <v>316</v>
       </c>
-      <c r="D242" s="24"/>
-      <c r="E242" s="24"/>
-      <c r="F242" s="24"/>
-      <c r="G242" s="24"/>
-      <c r="H242" s="24"/>
-      <c r="I242" s="24"/>
+      <c r="D242" s="25"/>
+      <c r="E242" s="25"/>
+      <c r="F242" s="25"/>
+      <c r="G242" s="25"/>
+      <c r="H242" s="25"/>
+      <c r="I242" s="25"/>
+    </row>
+    <row r="243" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A243" s="22" t="s">
+        <v>306</v>
+      </c>
+      <c r="B243" s="22"/>
+      <c r="C243" s="25" t="s">
+        <v>317</v>
+      </c>
+      <c r="D243" s="25"/>
+      <c r="E243" s="25"/>
+      <c r="F243" s="25"/>
+      <c r="G243" s="25"/>
+      <c r="H243" s="25"/>
+      <c r="I243" s="25"/>
+    </row>
+    <row r="244" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A244" s="22" t="s">
+        <v>306</v>
+      </c>
+      <c r="B244" s="22"/>
+      <c r="C244" s="25" t="s">
+        <v>318</v>
+      </c>
+      <c r="D244" s="25"/>
+      <c r="E244" s="25"/>
+      <c r="F244" s="25"/>
+      <c r="G244" s="25"/>
+      <c r="H244" s="25"/>
+      <c r="I244" s="25"/>
     </row>
   </sheetData>
-  <autoFilter ref="A5:I242"/>
-  <mergeCells count="14">
+  <autoFilter ref="A5:I244"/>
+  <mergeCells count="16">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A206:I206"/>
@@ -10435,6 +10476,8 @@
     <mergeCell ref="C240:I240"/>
     <mergeCell ref="C241:I241"/>
     <mergeCell ref="C242:I242"/>
+    <mergeCell ref="C243:I243"/>
+    <mergeCell ref="C244:I244"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>